<commit_message>
Generate clear inbound reservations locally and preserve ready attachments
</commit_message>
<xml_diff>
--- a/wecom-assistant/fixtures/inbound-template.xlsx
+++ b/wecom-assistant/fixtures/inbound-template.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="R5f3405b43f094892"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet2" sheetId="2" r:id="Rc49638723360474f"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="R307f720a0ec24661"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet2" sheetId="2" r:id="Rf17b5dbaed934f53"/>
   </sheets>
 </workbook>
 </file>
@@ -489,6 +489,30 @@
       </c>
       <c r="H7" t="str"/>
     </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>CWXXX0001</v>
+      </c>
+      <c r="B8" t="str">
+        <v>熊小小牛排饭-拌饭汁</v>
+      </c>
+      <c r="C8" t="str">
+        <v>CWXXX0001</v>
+      </c>
+      <c r="D8" t="str">
+        <v>常温</v>
+      </c>
+      <c r="E8" t="str">
+        <v>10kg/箱</v>
+      </c>
+      <c r="F8" t="str">
+        <v>整箱</v>
+      </c>
+      <c r="G8" t="str">
+        <v>件</v>
+      </c>
+      <c r="H8" t="str"/>
+    </row>
   </sheetData>
   <mergeCells>
     <mergeCell ref="B1:H1"/>

</xml_diff>